<commit_message>
Coherencia spec↔código: FCCJE, urbanización, CUEX, corrector de superficie y prefijo más largo
- traductor: errata FCCJS→FCCJE en regla de material de docencia (2236/2238)
- amortizaciones: regla «urbaniza»→urbanización en el rescate por descripción
- suministros/OTOP: reparto por prefijo más largo (zonas en exclusiva a la
  fila más específica) con pesos m²×corrector de superficie (energía+gas→
  corrector_energía, agua→corrección_otros, OTOP→corrección_limpieza)
- pod_no_oficial: filtro acepta CUEX (catálogo oficial), CUES como sinónimo
- spec: «no es 00» en investigación nacional, CUES→CUEX, ss-pi-otpersonal,
  correctores documentados, árbol de la app a ocho grupos y bloques nuevos
  del catálogo de pantallas, coana informes en entry points
- regeneradas salidas de fase 1, reparto e informes (cuadres Δ=0,
  conservación exacta)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/informes/cuadro_10_1.xlsx
+++ b/data/informes/cuadro_10_1.xlsx
@@ -525,7 +525,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.7630830000000001</v>
+        <v>0.762813</v>
       </c>
     </row>
     <row r="5">
@@ -736,7 +736,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>0.067982</v>
+        <v>0.067958</v>
       </c>
     </row>
     <row r="16">
@@ -871,7 +871,7 @@
         <v>1</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>0.10719</v>
+        <v>0.107152</v>
       </c>
     </row>
     <row r="23">
@@ -1061,13 +1061,13 @@
         </is>
       </c>
       <c r="C32" s="5" t="n">
-        <v>6347526.73</v>
+        <v>6401469.36</v>
       </c>
       <c r="D32" s="6" t="n">
         <v>1</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>0.041606</v>
+        <v>0.041944</v>
       </c>
     </row>
     <row r="33">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="C33" s="8" t="n">
-        <v>6347526.73</v>
+        <v>6401469.36</v>
       </c>
       <c r="D33" s="9" t="n">
         <v>1</v>
@@ -1147,7 +1147,7 @@
         <v>1</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>0.019938</v>
+        <v>0.019931</v>
       </c>
     </row>
     <row r="37">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="C40" s="11" t="n">
-        <v>152563950.4</v>
+        <v>152617893.03</v>
       </c>
       <c r="D40" s="10" t="n"/>
       <c r="E40" s="12" t="n">

</xml_diff>